<commit_message>
Se actualizan Visión del producto y requisitos
Solo un profesional de salud calificado puede confirmar o modificar el resultado del análisis. El encargado del gimnasio solo ve los resultados y deriva emergencias a atención médica.

Requisitos:
- R.104, R.105, R.119, R.230 y R.231: la revisión y la modificación del resultado quedan a cargo del profesional de salud.
- R.106 y R.138: el encargado deriva emergencias y esas derivaciones quedan registradas.
- R.172: el control de acceso por rol aplica esta regla.
- R.134 y R.232: se registran las modificaciones con su motivo y las derivaciones.
- Se agrega "Profesional de salud" como actor donde corresponde.

Visión del Producto:
- "Objetivos y métricas" refleja que el encargado ve resultados y deriva emergencias, sin confirmarlos.
- Edición de formato, métricas quedan en líneas separadas en vez de una línea junta.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Requisitos/Requisitos_Capstone_Thomas_Gutiérrez_Sebastián_Jara_Cristobal_Hernández.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Requisitos/Requisitos_Capstone_Thomas_Gutiérrez_Sebastián_Jara_Cristobal_Hernández.xlsx
@@ -634,7 +634,7 @@
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio, Administrador</t>
+          <t>Encargado del gimnasio, Profesional de salud, Administrador</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio, Administrador</t>
+          <t>Encargado del gimnasio, Profesional de salud, Administrador</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá restringir el acceso del dashboard según roles y permisos.</t>
+          <t>El sistema deberá restringir el acceso según el rol: el encargado solo ve resultados y deriva emergencias, y solo el profesional de salud puede modificar un resultado.</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Sistema, Encargado del gimnasio</t>
+          <t>Sistema, Profesional de salud, Encargado del gimnasio</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Equipo de datos, Encargado del gimnasio</t>
+          <t>Equipo de datos, Profesional de salud</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Equipo de datos, Encargado del gimnasio</t>
+          <t>Equipo de datos, Profesional de salud</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>IA, Encargado del gimnasio</t>
+          <t>IA, Profesional de salud</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -3917,12 +3917,12 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>La recomendación automática deberá poder ser revisada por el encargado del gimnasio.</t>
+          <t>La recomendación automática deberá poder ser revisada por un profesional de salud calificado.</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>No sustitución del criterio del encargado</t>
+          <t>No sustitución del criterio profesional</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -3949,12 +3949,12 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>IA, Encargado del gimnasio</t>
+          <t>IA, Profesional de salud</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá funcionar como apoyo a la decisión del encargado del gimnasio, nunca como reemplazo.</t>
+          <t>El sistema deberá funcionar como apoyo a la decisión: solo un profesional de salud calificado puede modificar el resultado.</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Registro de decisiones del encargado</t>
+          <t>Registro de decisiones</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -3981,12 +3981,12 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Sistema, Encargado del gimnasio</t>
+          <t>Sistema, Profesional de salud, Encargado del gimnasio</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá mantener trazabilidad de las decisiones tomadas por el encargado (confirmar o derivar).</t>
+          <t>El sistema deberá mantener trazabilidad de las decisiones del profesional de salud (confirmar o modificar) y de las derivaciones del encargado.</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Equipo de datos, Encargado del gimnasio</t>
+          <t>Equipo de datos, Profesional de salud</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Sistema, Encargado del gimnasio</t>
+          <t>Sistema, Profesional de salud</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -10455,12 +10455,12 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>IA, Encargado del gimnasio</t>
+          <t>IA, Profesional de salud</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá derivar las recomendaciones de baja confianza a revisión del encargado.</t>
+          <t>El sistema deberá derivar las recomendaciones de baja confianza a revisión de un profesional de salud.</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
@@ -10519,12 +10519,12 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir al encargado revisar la recomendación generada.</t>
+          <t>El sistema deberá permitir a un profesional de salud revisar la recomendación generada.</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -10541,7 +10541,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Confirmación de recomendación</t>
+          <t>Confirmación o modificación del resultado</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -10551,12 +10551,12 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir al encargado confirmar la recomendación sugerida.</t>
+          <t>El sistema deberá permitir que solo un profesional de salud calificado confirme o modifique el resultado del análisis.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
@@ -10573,7 +10573,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Derivación a evaluación médica</t>
+          <t>Derivación de emergencias</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -10588,7 +10588,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir al encargado derivar al usuario a evaluación médica en vez de confirmar la recomendación.</t>
+          <t>El sistema deberá permitir al encargado derivar al usuario a atención médica ante una emergencia.</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -10620,7 +10620,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar el motivo de cada derivación.</t>
+          <t>El sistema deberá registrar el motivo de cada derivación de emergencia.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -10701,7 +10701,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Comparación IA-Encargado</t>
+          <t>Comparación IA-Profesional</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -10711,12 +10711,12 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>IA, Encargado del gimnasio</t>
+          <t>IA, Profesional de salud</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir comparar la recomendación de la IA con la decisión final del encargado.</t>
+          <t>El sistema deberá permitir comparar la recomendación de la IA con la decisión final del profesional de salud.</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -10807,12 +10807,12 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>IA, Encargado del gimnasio</t>
+          <t>IA, Profesional de salud</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá derivar al encargado cuando no exista información suficiente para recomendar.</t>
+          <t>El sistema deberá derivar a revisión de un profesional de salud cuando no exista información suficiente para recomendar.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
@@ -10999,12 +10999,12 @@
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Sistema, Encargado del gimnasio</t>
+          <t>Sistema, Profesional de salud</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar la decisión final del encargado: confirmar o derivar.</t>
+          <t>El sistema deberá registrar la decisión final del profesional de salud: confirmar o modificar el resultado.</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -11678,12 +11678,12 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir al encargado registrar observaciones.</t>
+          <t>El sistema deberá permitir al profesional de salud registrar observaciones.</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -11806,12 +11806,12 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar la confirmación hecha por el encargado.</t>
+          <t>El sistema deberá registrar la confirmación hecha por el profesional de salud.</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -11828,7 +11828,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Registro de rechazo de recomendación</t>
+          <t>Registro de modificación del resultado</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -11838,12 +11838,12 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar cuando el encargado no esté de acuerdo con la recomendación y derive al usuario.</t>
+          <t>El sistema deberá registrar cuando un profesional de salud modifique el resultado, junto con el motivo.</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -11870,12 +11870,12 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá permitir gestionar la lista de evaluaciones pendientes de revisión.</t>
+          <t>El sistema deberá permitir al profesional de salud gestionar la lista de evaluaciones pendientes de revisión.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud, Encargado del gimnasio</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -11934,12 +11934,12 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Encargado del gimnasio</t>
+          <t>Profesional de salud</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar cuando una evaluación haya sido revisada.</t>
+          <t>El sistema deberá registrar cuando un profesional de salud haya revisado una evaluación.</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -11971,7 +11971,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>El sistema deberá registrar cuando un usuario sea derivado a evaluación médica externa.</t>
+          <t>El sistema deberá registrar cuando el encargado derive a un usuario a atención médica.</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">

</xml_diff>